<commit_message>
Reto y kit: fechas reales (lunes 19/10, 11 dias habiles), inscrito pagado definido sin porcentajes, sin regla de base de datos, una sola fecha de inicio (3/11), clases sin 'ingles desde el dia 1' ni simulaciones, grupos de maximo 16, Modulo de Graduacion y condiciones de la garantia ampliados, plan empresa desde 3 cupos
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/FORMATO_15_EMPRESAS_RETO.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/FORMATO_15_EMPRESAS_RETO.xlsx
@@ -1069,7 +1069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1122,7 +1122,7 @@
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="6" t="n">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="B5" s="5" t="n"/>
       <c r="C5" s="5" t="n"/>
@@ -1131,7 +1131,7 @@
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="9" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="B6" s="8" t="n"/>
       <c r="C6" s="8" t="n"/>
@@ -1140,7 +1140,7 @@
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="6" t="n">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="B7" s="5" t="n"/>
       <c r="C7" s="5" t="n"/>
@@ -1149,7 +1149,7 @@
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="9" t="n">
-        <v>46318</v>
+        <v>46317</v>
       </c>
       <c r="B8" s="8" t="n"/>
       <c r="C8" s="8" t="n"/>
@@ -1158,7 +1158,7 @@
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="6" t="n">
-        <v>46321</v>
+        <v>46318</v>
       </c>
       <c r="B9" s="5" t="n"/>
       <c r="C9" s="5" t="n"/>
@@ -1167,7 +1167,7 @@
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="9" t="n">
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="B10" s="8" t="n"/>
       <c r="C10" s="8" t="n"/>
@@ -1176,7 +1176,7 @@
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="6" t="n">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="5" t="n"/>
@@ -1185,7 +1185,7 @@
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="9" t="n">
-        <v>46324</v>
+        <v>46323</v>
       </c>
       <c r="B12" s="8" t="n"/>
       <c r="C12" s="8" t="n"/>
@@ -1194,7 +1194,7 @@
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="6" t="n">
-        <v>46325</v>
+        <v>46324</v>
       </c>
       <c r="B13" s="5" t="n"/>
       <c r="C13" s="5" t="n"/>
@@ -1203,74 +1203,83 @@
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="9" t="n">
-        <v>46328</v>
+        <v>46325</v>
       </c>
       <c r="B14" s="8" t="n"/>
       <c r="C14" s="8" t="n"/>
       <c r="D14" s="8" t="n"/>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>Festivo: sin contacto a clientes</t>
-        </is>
-      </c>
+      <c r="E14" s="8" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="6" t="n">
-        <v>46329</v>
+        <v>46328</v>
       </c>
       <c r="B15" s="5" t="n"/>
       <c r="C15" s="5" t="n"/>
       <c r="D15" s="5" t="n"/>
       <c r="E15" s="5" t="inlineStr">
         <is>
+          <t>Festivo: sin contacto a clientes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="9" t="n">
+        <v>46329</v>
+      </c>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
           <t>CORTE 6:00 p. m.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B16" s="11">
-        <f>SUM(B5:B15)</f>
+      <c r="B17" s="11">
+        <f>SUM(B5:B16)</f>
         <v/>
       </c>
-      <c r="C16" s="11">
-        <f>SUM(C5:C15)</f>
+      <c r="C17" s="11">
+        <f>SUM(C5:C16)</f>
         <v/>
       </c>
-      <c r="D16" s="11">
-        <f>MAX(D5:D15)</f>
+      <c r="D17" s="11">
+        <f>MAX(D5:D16)</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>Ritmo mínimo</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>Mar 21/10: 15 empresas contactadas con el decisor (acumulado).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>Vie 24/10: 8 reuniones con decisor y 3 charlas autorizadas para la semana 2.</t>
+          <t>Mar 20/10: 15 empresas contactadas con el decisor (acumulado).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>Mar 3/11, 6:00 p. m.: 10 inscritos pagados, al menos 5 de una misma empresa.</t>
+          <t>Vie 23/10: 8 reuniones con decisor y 3 charlas autorizadas para la semana 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>Mar 3/11, 6:00 p. m.: 10 inscritos pagados.</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1288,7 @@
     <mergeCell ref="A2:E2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B5:D15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Número entero." type="whole" operator="greaterThanOrEqual">
+    <dataValidation sqref="B5:D16" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Número entero." type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Reto: meta 10 inscritos pagados o 30M en caja (lo que llegue primero), cualquier programa; Excel con caja acumulada; 8:30
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/FORMATO_15_EMPRESAS_RETO.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/FORMATO_15_EMPRESAS_RETO.xlsx
@@ -106,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -136,6 +136,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -534,7 +541,7 @@
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Toda empresa se registra aquí ANTES de la primera reunión. Empresas de 40 a 150 empleados donde el dueño o el gerente decide. Planilla al día antes de la llamada de las 8:00 a. m. Uso interno: los datos no se comparten.</t>
+          <t>Toda empresa se registra aquí ANTES de la primera reunión. Empresas de 40 a 150 empleados donde el dueño o el gerente decide. Planilla al día antes de la llamada de las 8:30 a. m. Uso interno: los datos no se comparten.</t>
         </is>
       </c>
     </row>
@@ -1069,27 +1076,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REPORTE DIARIO · se llena antes de la llamada de las 8:00 a. m.</t>
+          <t>REPORTE DIARIO · se llena antes de la llamada de las 8:30 a. m.</t>
         </is>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tres líneas por día. Inscritos pagados = inicial en la cuenta de Heiiu, verificada por coordinación. Corte: martes 3/11 a las 6:00 p. m. El lunes 2/11 es festivo.</t>
+          <t>Cuatro datos por día. Inscritos pagados = contado, o inicial más contrato firmado. Caja = dinero verificado en la cuenta de Heiiu. Meta: 10 inscritos o $30.000.000, lo que llegue primero. Corte: martes 3/11 a las 6:00 p. m. El lunes 2/11 es festivo.</t>
         </is>
       </c>
     </row>
@@ -1115,6 +1123,11 @@
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Caja acumulada ($)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Nota del día (1 línea)</t>
         </is>
@@ -1127,7 +1140,8 @@
       <c r="B5" s="5" t="n"/>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
+      <c r="E5" s="13" t="n"/>
+      <c r="F5" s="5" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="9" t="n">
@@ -1136,7 +1150,8 @@
       <c r="B6" s="8" t="n"/>
       <c r="C6" s="8" t="n"/>
       <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
+      <c r="E6" s="14" t="n"/>
+      <c r="F6" s="8" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="6" t="n">
@@ -1145,7 +1160,8 @@
       <c r="B7" s="5" t="n"/>
       <c r="C7" s="5" t="n"/>
       <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
+      <c r="E7" s="13" t="n"/>
+      <c r="F7" s="5" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="9" t="n">
@@ -1154,7 +1170,8 @@
       <c r="B8" s="8" t="n"/>
       <c r="C8" s="8" t="n"/>
       <c r="D8" s="8" t="n"/>
-      <c r="E8" s="8" t="n"/>
+      <c r="E8" s="14" t="n"/>
+      <c r="F8" s="8" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="6" t="n">
@@ -1163,7 +1180,8 @@
       <c r="B9" s="5" t="n"/>
       <c r="C9" s="5" t="n"/>
       <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
+      <c r="E9" s="13" t="n"/>
+      <c r="F9" s="5" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="9" t="n">
@@ -1172,7 +1190,8 @@
       <c r="B10" s="8" t="n"/>
       <c r="C10" s="8" t="n"/>
       <c r="D10" s="8" t="n"/>
-      <c r="E10" s="8" t="n"/>
+      <c r="E10" s="14" t="n"/>
+      <c r="F10" s="8" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -1181,7 +1200,8 @@
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="5" t="n"/>
       <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
+      <c r="E11" s="13" t="n"/>
+      <c r="F11" s="5" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="9" t="n">
@@ -1190,7 +1210,8 @@
       <c r="B12" s="8" t="n"/>
       <c r="C12" s="8" t="n"/>
       <c r="D12" s="8" t="n"/>
-      <c r="E12" s="8" t="n"/>
+      <c r="E12" s="14" t="n"/>
+      <c r="F12" s="8" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -1199,7 +1220,8 @@
       <c r="B13" s="5" t="n"/>
       <c r="C13" s="5" t="n"/>
       <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
+      <c r="E13" s="13" t="n"/>
+      <c r="F13" s="5" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="9" t="n">
@@ -1208,7 +1230,8 @@
       <c r="B14" s="8" t="n"/>
       <c r="C14" s="8" t="n"/>
       <c r="D14" s="8" t="n"/>
-      <c r="E14" s="8" t="n"/>
+      <c r="E14" s="14" t="n"/>
+      <c r="F14" s="8" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -1217,7 +1240,8 @@
       <c r="B15" s="5" t="n"/>
       <c r="C15" s="5" t="n"/>
       <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="13" t="n"/>
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Festivo: sin contacto a clientes</t>
         </is>
@@ -1230,7 +1254,8 @@
       <c r="B16" s="8" t="n"/>
       <c r="C16" s="8" t="n"/>
       <c r="D16" s="8" t="n"/>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E16" s="14" t="n"/>
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>CORTE 6:00 p. m.</t>
         </is>
@@ -1254,6 +1279,10 @@
         <f>MAX(D5:D16)</f>
         <v/>
       </c>
+      <c r="E17" s="15">
+        <f>MAX(E5:E16)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
@@ -1279,13 +1308,13 @@
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>Mar 3/11, 6:00 p. m.: 10 inscritos pagados.</t>
+          <t>Mar 3/11, 6:00 p. m.: 10 inscritos pagados o $30.000.000 en caja, lo que llegue primero.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A2:F2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="B5:D16" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Número entero." type="whole" operator="greaterThanOrEqual">
@@ -1322,7 +1351,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Empresa: ______________________________   Fecha de la charla: ____ / ____ / 2026</t>
         </is>
@@ -1376,276 +1405,276 @@
       <c r="A6" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="14" t="n"/>
-      <c r="C6" s="14" t="n"/>
-      <c r="D6" s="14" t="n"/>
-      <c r="E6" s="14" t="n"/>
-      <c r="F6" s="14" t="n"/>
-      <c r="G6" s="14" t="n"/>
+      <c r="B6" s="17" t="n"/>
+      <c r="C6" s="17" t="n"/>
+      <c r="D6" s="17" t="n"/>
+      <c r="E6" s="17" t="n"/>
+      <c r="F6" s="17" t="n"/>
+      <c r="G6" s="17" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="15" t="n"/>
-      <c r="C7" s="15" t="n"/>
-      <c r="D7" s="15" t="n"/>
-      <c r="E7" s="15" t="n"/>
-      <c r="F7" s="15" t="n"/>
-      <c r="G7" s="15" t="n"/>
+      <c r="B7" s="18" t="n"/>
+      <c r="C7" s="18" t="n"/>
+      <c r="D7" s="18" t="n"/>
+      <c r="E7" s="18" t="n"/>
+      <c r="F7" s="18" t="n"/>
+      <c r="G7" s="18" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="14" t="n"/>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="14" t="n"/>
-      <c r="E8" s="14" t="n"/>
-      <c r="F8" s="14" t="n"/>
-      <c r="G8" s="14" t="n"/>
+      <c r="B8" s="17" t="n"/>
+      <c r="C8" s="17" t="n"/>
+      <c r="D8" s="17" t="n"/>
+      <c r="E8" s="17" t="n"/>
+      <c r="F8" s="17" t="n"/>
+      <c r="G8" s="17" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="15" t="n"/>
-      <c r="C9" s="15" t="n"/>
-      <c r="D9" s="15" t="n"/>
-      <c r="E9" s="15" t="n"/>
-      <c r="F9" s="15" t="n"/>
-      <c r="G9" s="15" t="n"/>
+      <c r="B9" s="18" t="n"/>
+      <c r="C9" s="18" t="n"/>
+      <c r="D9" s="18" t="n"/>
+      <c r="E9" s="18" t="n"/>
+      <c r="F9" s="18" t="n"/>
+      <c r="G9" s="18" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="14" t="n"/>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="14" t="n"/>
-      <c r="E10" s="14" t="n"/>
-      <c r="F10" s="14" t="n"/>
-      <c r="G10" s="14" t="n"/>
+      <c r="B10" s="17" t="n"/>
+      <c r="C10" s="17" t="n"/>
+      <c r="D10" s="17" t="n"/>
+      <c r="E10" s="17" t="n"/>
+      <c r="F10" s="17" t="n"/>
+      <c r="G10" s="17" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="15" t="n"/>
-      <c r="C11" s="15" t="n"/>
-      <c r="D11" s="15" t="n"/>
-      <c r="E11" s="15" t="n"/>
-      <c r="F11" s="15" t="n"/>
-      <c r="G11" s="15" t="n"/>
+      <c r="B11" s="18" t="n"/>
+      <c r="C11" s="18" t="n"/>
+      <c r="D11" s="18" t="n"/>
+      <c r="E11" s="18" t="n"/>
+      <c r="F11" s="18" t="n"/>
+      <c r="G11" s="18" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="14" t="n"/>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="14" t="n"/>
-      <c r="E12" s="14" t="n"/>
-      <c r="F12" s="14" t="n"/>
-      <c r="G12" s="14" t="n"/>
+      <c r="B12" s="17" t="n"/>
+      <c r="C12" s="17" t="n"/>
+      <c r="D12" s="17" t="n"/>
+      <c r="E12" s="17" t="n"/>
+      <c r="F12" s="17" t="n"/>
+      <c r="G12" s="17" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="15" t="n"/>
-      <c r="C13" s="15" t="n"/>
-      <c r="D13" s="15" t="n"/>
-      <c r="E13" s="15" t="n"/>
-      <c r="F13" s="15" t="n"/>
-      <c r="G13" s="15" t="n"/>
+      <c r="B13" s="18" t="n"/>
+      <c r="C13" s="18" t="n"/>
+      <c r="D13" s="18" t="n"/>
+      <c r="E13" s="18" t="n"/>
+      <c r="F13" s="18" t="n"/>
+      <c r="G13" s="18" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="14" t="n"/>
-      <c r="C14" s="14" t="n"/>
-      <c r="D14" s="14" t="n"/>
-      <c r="E14" s="14" t="n"/>
-      <c r="F14" s="14" t="n"/>
-      <c r="G14" s="14" t="n"/>
+      <c r="B14" s="17" t="n"/>
+      <c r="C14" s="17" t="n"/>
+      <c r="D14" s="17" t="n"/>
+      <c r="E14" s="17" t="n"/>
+      <c r="F14" s="17" t="n"/>
+      <c r="G14" s="17" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="15" t="n"/>
-      <c r="C15" s="15" t="n"/>
-      <c r="D15" s="15" t="n"/>
-      <c r="E15" s="15" t="n"/>
-      <c r="F15" s="15" t="n"/>
-      <c r="G15" s="15" t="n"/>
+      <c r="B15" s="18" t="n"/>
+      <c r="C15" s="18" t="n"/>
+      <c r="D15" s="18" t="n"/>
+      <c r="E15" s="18" t="n"/>
+      <c r="F15" s="18" t="n"/>
+      <c r="G15" s="18" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="14" t="n"/>
-      <c r="C16" s="14" t="n"/>
-      <c r="D16" s="14" t="n"/>
-      <c r="E16" s="14" t="n"/>
-      <c r="F16" s="14" t="n"/>
-      <c r="G16" s="14" t="n"/>
+      <c r="B16" s="17" t="n"/>
+      <c r="C16" s="17" t="n"/>
+      <c r="D16" s="17" t="n"/>
+      <c r="E16" s="17" t="n"/>
+      <c r="F16" s="17" t="n"/>
+      <c r="G16" s="17" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B17" s="15" t="n"/>
-      <c r="C17" s="15" t="n"/>
-      <c r="D17" s="15" t="n"/>
-      <c r="E17" s="15" t="n"/>
-      <c r="F17" s="15" t="n"/>
-      <c r="G17" s="15" t="n"/>
+      <c r="B17" s="18" t="n"/>
+      <c r="C17" s="18" t="n"/>
+      <c r="D17" s="18" t="n"/>
+      <c r="E17" s="18" t="n"/>
+      <c r="F17" s="18" t="n"/>
+      <c r="G17" s="18" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B18" s="14" t="n"/>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="14" t="n"/>
-      <c r="E18" s="14" t="n"/>
-      <c r="F18" s="14" t="n"/>
-      <c r="G18" s="14" t="n"/>
+      <c r="B18" s="17" t="n"/>
+      <c r="C18" s="17" t="n"/>
+      <c r="D18" s="17" t="n"/>
+      <c r="E18" s="17" t="n"/>
+      <c r="F18" s="17" t="n"/>
+      <c r="G18" s="17" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="B19" s="15" t="n"/>
-      <c r="C19" s="15" t="n"/>
-      <c r="D19" s="15" t="n"/>
-      <c r="E19" s="15" t="n"/>
-      <c r="F19" s="15" t="n"/>
-      <c r="G19" s="15" t="n"/>
+      <c r="B19" s="18" t="n"/>
+      <c r="C19" s="18" t="n"/>
+      <c r="D19" s="18" t="n"/>
+      <c r="E19" s="18" t="n"/>
+      <c r="F19" s="18" t="n"/>
+      <c r="G19" s="18" t="n"/>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B20" s="14" t="n"/>
-      <c r="C20" s="14" t="n"/>
-      <c r="D20" s="14" t="n"/>
-      <c r="E20" s="14" t="n"/>
-      <c r="F20" s="14" t="n"/>
-      <c r="G20" s="14" t="n"/>
+      <c r="B20" s="17" t="n"/>
+      <c r="C20" s="17" t="n"/>
+      <c r="D20" s="17" t="n"/>
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="17" t="n"/>
+      <c r="G20" s="17" t="n"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="B21" s="15" t="n"/>
-      <c r="C21" s="15" t="n"/>
-      <c r="D21" s="15" t="n"/>
-      <c r="E21" s="15" t="n"/>
-      <c r="F21" s="15" t="n"/>
-      <c r="G21" s="15" t="n"/>
+      <c r="B21" s="18" t="n"/>
+      <c r="C21" s="18" t="n"/>
+      <c r="D21" s="18" t="n"/>
+      <c r="E21" s="18" t="n"/>
+      <c r="F21" s="18" t="n"/>
+      <c r="G21" s="18" t="n"/>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B22" s="14" t="n"/>
-      <c r="C22" s="14" t="n"/>
-      <c r="D22" s="14" t="n"/>
-      <c r="E22" s="14" t="n"/>
-      <c r="F22" s="14" t="n"/>
-      <c r="G22" s="14" t="n"/>
+      <c r="B22" s="17" t="n"/>
+      <c r="C22" s="17" t="n"/>
+      <c r="D22" s="17" t="n"/>
+      <c r="E22" s="17" t="n"/>
+      <c r="F22" s="17" t="n"/>
+      <c r="G22" s="17" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="B23" s="15" t="n"/>
-      <c r="C23" s="15" t="n"/>
-      <c r="D23" s="15" t="n"/>
-      <c r="E23" s="15" t="n"/>
-      <c r="F23" s="15" t="n"/>
-      <c r="G23" s="15" t="n"/>
+      <c r="B23" s="18" t="n"/>
+      <c r="C23" s="18" t="n"/>
+      <c r="D23" s="18" t="n"/>
+      <c r="E23" s="18" t="n"/>
+      <c r="F23" s="18" t="n"/>
+      <c r="G23" s="18" t="n"/>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B24" s="14" t="n"/>
-      <c r="C24" s="14" t="n"/>
-      <c r="D24" s="14" t="n"/>
-      <c r="E24" s="14" t="n"/>
-      <c r="F24" s="14" t="n"/>
-      <c r="G24" s="14" t="n"/>
+      <c r="B24" s="17" t="n"/>
+      <c r="C24" s="17" t="n"/>
+      <c r="D24" s="17" t="n"/>
+      <c r="E24" s="17" t="n"/>
+      <c r="F24" s="17" t="n"/>
+      <c r="G24" s="17" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="B25" s="15" t="n"/>
-      <c r="C25" s="15" t="n"/>
-      <c r="D25" s="15" t="n"/>
-      <c r="E25" s="15" t="n"/>
-      <c r="F25" s="15" t="n"/>
-      <c r="G25" s="15" t="n"/>
+      <c r="B25" s="18" t="n"/>
+      <c r="C25" s="18" t="n"/>
+      <c r="D25" s="18" t="n"/>
+      <c r="E25" s="18" t="n"/>
+      <c r="F25" s="18" t="n"/>
+      <c r="G25" s="18" t="n"/>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="B26" s="14" t="n"/>
-      <c r="C26" s="14" t="n"/>
-      <c r="D26" s="14" t="n"/>
-      <c r="E26" s="14" t="n"/>
-      <c r="F26" s="14" t="n"/>
-      <c r="G26" s="14" t="n"/>
+      <c r="B26" s="17" t="n"/>
+      <c r="C26" s="17" t="n"/>
+      <c r="D26" s="17" t="n"/>
+      <c r="E26" s="17" t="n"/>
+      <c r="F26" s="17" t="n"/>
+      <c r="G26" s="17" t="n"/>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="7" t="n">
         <v>22</v>
       </c>
-      <c r="B27" s="15" t="n"/>
-      <c r="C27" s="15" t="n"/>
-      <c r="D27" s="15" t="n"/>
-      <c r="E27" s="15" t="n"/>
-      <c r="F27" s="15" t="n"/>
-      <c r="G27" s="15" t="n"/>
+      <c r="B27" s="18" t="n"/>
+      <c r="C27" s="18" t="n"/>
+      <c r="D27" s="18" t="n"/>
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="18" t="n"/>
+      <c r="G27" s="18" t="n"/>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="B28" s="14" t="n"/>
-      <c r="C28" s="14" t="n"/>
-      <c r="D28" s="14" t="n"/>
-      <c r="E28" s="14" t="n"/>
-      <c r="F28" s="14" t="n"/>
-      <c r="G28" s="14" t="n"/>
+      <c r="B28" s="17" t="n"/>
+      <c r="C28" s="17" t="n"/>
+      <c r="D28" s="17" t="n"/>
+      <c r="E28" s="17" t="n"/>
+      <c r="F28" s="17" t="n"/>
+      <c r="G28" s="17" t="n"/>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="B29" s="15" t="n"/>
-      <c r="C29" s="15" t="n"/>
-      <c r="D29" s="15" t="n"/>
-      <c r="E29" s="15" t="n"/>
-      <c r="F29" s="15" t="n"/>
-      <c r="G29" s="15" t="n"/>
+      <c r="B29" s="18" t="n"/>
+      <c r="C29" s="18" t="n"/>
+      <c r="D29" s="18" t="n"/>
+      <c r="E29" s="18" t="n"/>
+      <c r="F29" s="18" t="n"/>
+      <c r="G29" s="18" t="n"/>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="B30" s="14" t="n"/>
-      <c r="C30" s="14" t="n"/>
-      <c r="D30" s="14" t="n"/>
-      <c r="E30" s="14" t="n"/>
-      <c r="F30" s="14" t="n"/>
-      <c r="G30" s="14" t="n"/>
+      <c r="B30" s="17" t="n"/>
+      <c r="C30" s="17" t="n"/>
+      <c r="D30" s="17" t="n"/>
+      <c r="E30" s="17" t="n"/>
+      <c r="F30" s="17" t="n"/>
+      <c r="G30" s="17" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Reto de arranque para el candidato 3 (arranque miercoles 21/10, 9 dias habiles); kit, Excel y hoja de induccion con fechas del miercoles 21
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/FORMATO_15_EMPRESAS_RETO.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/FORMATO_15_EMPRESAS_RETO.xlsx
@@ -1076,7 +1076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1135,7 +1135,7 @@
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="6" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
       <c r="B5" s="5" t="n"/>
       <c r="C5" s="5" t="n"/>
@@ -1145,7 +1145,7 @@
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="9" t="n">
-        <v>46315</v>
+        <v>46317</v>
       </c>
       <c r="B6" s="8" t="n"/>
       <c r="C6" s="8" t="n"/>
@@ -1155,7 +1155,7 @@
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="6" t="n">
-        <v>46316</v>
+        <v>46318</v>
       </c>
       <c r="B7" s="5" t="n"/>
       <c r="C7" s="5" t="n"/>
@@ -1165,7 +1165,7 @@
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="9" t="n">
-        <v>46317</v>
+        <v>46321</v>
       </c>
       <c r="B8" s="8" t="n"/>
       <c r="C8" s="8" t="n"/>
@@ -1175,7 +1175,7 @@
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="6" t="n">
-        <v>46318</v>
+        <v>46322</v>
       </c>
       <c r="B9" s="5" t="n"/>
       <c r="C9" s="5" t="n"/>
@@ -1185,7 +1185,7 @@
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="9" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
       <c r="B10" s="8" t="n"/>
       <c r="C10" s="8" t="n"/>
@@ -1195,7 +1195,7 @@
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="6" t="n">
-        <v>46322</v>
+        <v>46324</v>
       </c>
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="5" t="n"/>
@@ -1205,7 +1205,7 @@
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="9" t="n">
-        <v>46323</v>
+        <v>46325</v>
       </c>
       <c r="B12" s="8" t="n"/>
       <c r="C12" s="8" t="n"/>
@@ -1215,98 +1215,78 @@
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="6" t="n">
-        <v>46324</v>
+        <v>46328</v>
       </c>
       <c r="B13" s="5" t="n"/>
       <c r="C13" s="5" t="n"/>
       <c r="D13" s="5" t="n"/>
       <c r="E13" s="13" t="n"/>
-      <c r="F13" s="5" t="n"/>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Festivo: sin contacto a clientes</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="9" t="n">
-        <v>46325</v>
+        <v>46329</v>
       </c>
       <c r="B14" s="8" t="n"/>
       <c r="C14" s="8" t="n"/>
       <c r="D14" s="8" t="n"/>
       <c r="E14" s="14" t="n"/>
-      <c r="F14" s="8" t="n"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="6" t="n">
-        <v>46328</v>
-      </c>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="13" t="n"/>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>Festivo: sin contacto a clientes</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="9" t="n">
-        <v>46329</v>
-      </c>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="14" t="n"/>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>CORTE 6:00 p. m.</t>
         </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B15" s="11">
+        <f>SUM(B5:B14)</f>
+        <v/>
+      </c>
+      <c r="C15" s="11">
+        <f>SUM(C5:C14)</f>
+        <v/>
+      </c>
+      <c r="D15" s="11">
+        <f>MAX(D5:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="15">
+        <f>MAX(E5:E14)</f>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B17" s="11">
-        <f>SUM(B5:B16)</f>
-        <v/>
-      </c>
-      <c r="C17" s="11">
-        <f>SUM(C5:C16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="11">
-        <f>MAX(D5:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="15">
-        <f>MAX(E5:E16)</f>
-        <v/>
+          <t>Ritmo mínimo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Jue 22/10: 15 empresas contactadas con el decisor (acumulado).</t>
+        </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>Ritmo mínimo</t>
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Mar 27/10: 8 reuniones con decisor y 3 charlas autorizadas para la semana 2.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>Mar 20/10: 15 empresas contactadas con el decisor (acumulado).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>Vie 23/10: 8 reuniones con decisor y 3 charlas autorizadas para la semana 2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>Mar 3/11, 6:00 p. m.: 10 inscritos pagados o $30.000.000 en caja, lo que llegue primero.</t>
         </is>
@@ -1317,7 +1297,7 @@
     <mergeCell ref="A2:F2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B5:D16" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Número entero." type="whole" operator="greaterThanOrEqual">
+    <dataValidation sqref="B5:D14" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Número entero." type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>